<commit_message>
[EXECUTOR] xlsx 12-sheet + RULE_FREEZE v2.0 — Case_01
Sprint 6: traceability matrix expanded from 10 to 12 sheets; RULE_FREEZE v2.0.
- 22_Traceability_Matrix.xlsx: 2 new sheets — FUNCUC_TO_SECUC (35 constrains edges) + MUC_TO_MITIGATION (8 MUC rows). Total: 12 sheets.
- Script extended with FUNCTIONAL_UC_FREEZE (23), MUC_FREEZE (8), CONSTRAINS_EDGES (35) constants; coverage_dashboard adds 4 new metrics.
- RULE_FREEZE v2.0: §5 UC enumeration extended; v1.0 35 security U.C.s preserved verbatim; +23 functional U.C.s (PKG-7..11) + 8 MUCs documented. F-S5-02 marked RESOLVED.
- KG E4 incremental rebuild (Deucalion, ~14h) logged as follow-up — human approval required (P7).
- Counts: 46 rules / 35 sec U.C. / 23 func U.C. / 8 MUC / 30 FR / 46 NFR / 30 gates / 49 nodes / 10 risks / 38 threats.
</commit_message>
<xml_diff>
--- a/02_CASES/Case_01_TinyTask_SaaS/03_PHASE3_DECOMPOSITION_RICH/22_Traceability_Matrix.xlsx
+++ b/02_CASES/Case_01_TinyTask_SaaS/03_PHASE3_DECOMPOSITION_RICH/22_Traceability_Matrix.xlsx
@@ -17,6 +17,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COVERAGE_DASHBOARD" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RULE_FREEZE" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KG_CHAINS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FUNCUC_TO_SECUC" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MUC_TO_MITIGATION" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,10 +441,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -526,7 +528,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CORPUS_ENRICHED (Sprint 3 — placeholder cells; Sprint 5 deep-fills)</t>
+          <t>REWRITTEN_PRODUCT_BASELINE (Sprint 6 — 35 security U.C. + 23 functional U.C. + 8 MUCs)</t>
         </is>
       </c>
     </row>
@@ -538,7 +540,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -550,7 +552,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -562,7 +564,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-24 10:49 UTC</t>
+          <t>2026-08-26 15:30 UTC</t>
         </is>
       </c>
     </row>
@@ -598,110 +600,110 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>03_PHASE3_DECOMPOSITION_RICH/RULE_FREEZE.md (Sprint 1 frozen)</t>
+          <t>03_PHASE3_DECOMPOSITION_RICH/RULE_FREEZE.md v2.0 (Sprint 6 frozen)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Corpus linkage</t>
+          <t>Source of truth — UC catalog</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>03_PHASE3_DECOMPOSITION_RICH/CORPUS_LINKAGE.md (344 artefacts)</t>
+          <t>03_PHASE3_DECOMPOSITION_RICH/Doc20_Use_Cases_Catalog.md v3.0 (35 SEC + 23 FUNC + 8 MUC)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>NIST anchors</t>
+          <t>Source of truth — Relationships</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>03_PHASE3_DECOMPOSITION_RICH/NIST_ANCHORS.md (46 rules + 31 goals)</t>
+          <t>03_PHASE3_DECOMPOSITION_RICH/Doc21_Use_Case_Relationships.md v1.0 (91 edges)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>KG chains</t>
+          <t>Source of truth — Variability</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>03_PHASE3_DECOMPOSITION_RICH/KG_CHAINS.md (12 chains)</t>
+          <t>03_PHASE3_DECOMPOSITION_RICH/Doc22_Use_Case_Variability.md v1.0 (26 variants)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Total Sheets</t>
+          <t>Corpus linkage</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>03_PHASE3_DECOMPOSITION_RICH/CORPUS_LINKAGE.md (344 artefacts)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Sheets</t>
+          <t>NIST anchors</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>COVER, FULL_TRACEABILITY, NFR_TO_FR, FR_TO_UC, UC_TO_REGULATION, RULES_SATISFACTION, GATES_STATUS, COVERAGE_DASHBOARD, RULE_FREEZE, KG_CHAINS</t>
+          <t>03_PHASE3_DECOMPOSITION_RICH/NIST_ANCHORS.md (46 rules + 31 goals)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Freeze — Rules (CR + BPR)</t>
+          <t>KG chains</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>03_PHASE3_DECOMPOSITION_RICH/KG_CHAINS.md (12 chains; KG E4 incremental rebuild logged as follow-up)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Freeze — UCs (L1 cards)</t>
+          <t>Total Sheets</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Freeze — FRs</t>
+          <t>Sheets</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>COVER, FULL_TRACEABILITY, NFR_TO_FR, FR_TO_UC, UC_TO_REGULATION, RULES_SATISFACTION, GATES_STATUS, COVERAGE_DASHBOARD, RULE_FREEZE, KG_CHAINS, FUNCUC_TO_SECUC, MUC_TO_MITIGATION</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Freeze — NFRs</t>
+          <t>Freeze — Rules (CR + BPR)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -713,82 +715,166 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Freeze — Gates</t>
+          <t>Freeze — Security U.C.s (L1)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>35</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Freeze — Nodes</t>
+          <t>Freeze — Functional U.C.s (new)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>23</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Freeze — Risks + Threats</t>
+          <t>Freeze — MUCs (new)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10 + 38</t>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Generator script</t>
+          <t>Freeze — FRs</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>scripts/build_traceability_matrix_rich.py</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Validator script (light)</t>
+          <t>Freeze — NFRs</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>scripts/verify_rich.py (verify_xlsx() real; full verify Sprint 5)</t>
+          <t>46</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Author</t>
+          <t>Freeze — Gates</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sprint 3 Executor (paulo@methodology.pt)</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>Freeze — Nodes</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Freeze — Risks + Threats</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10 + 38</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Freeze — Constrains edges</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Freeze — MUC mitigations</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Generator script</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>scripts/build_traceability_matrix_rich.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Validator script (light)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>scripts/verify_rich.py (verify_xlsx() real; full verify Sprint 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Sprint 6 Executor (paulo@methodology.pt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>feature/aegis-p3-case01-rich</t>
         </is>
@@ -1355,6 +1441,1042 @@
       <c r="I13" t="inlineStr">
         <is>
           <t>PARSED</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Security UC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Constrains Functional UC(s)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Constraint type</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>U.C.1.1.1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>U.C.11.1.1, U.C.11.2.1, U.C.11.3.1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Rights enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>U.C.1.1.2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>U.C.11.1.1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Rights enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>U.C.1.2.1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>U.C.11.3.1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Rights enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>U.C.1.3.1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>U.C.11.2.1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Rights enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>U.C.1.4.1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>U.C.7.1.1, U.C.11.1.1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Rights enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>U.C.1.5.1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>U.C.11.2.1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Rights enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>U.C.2.1.1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>U.C.8.2.1, U.C.9.3.1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Availability / release gating</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>U.C.2.2.1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Availability / release gating</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>U.C.2.3.1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Availability / release gating</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>U.C.2.4.1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>U.C.8.2.1, U.C.9.3.1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Availability / release gating</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>U.C.2.4.2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Availability / release gating</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>U.C.2.5.1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Availability / release gating</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>U.C.2.6.1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Availability / release gating</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>U.C.3.1.1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>U.C.7.1.1, U.C.7.1.2, U.C.7.1.3, U.C.7.2.1, U.C.10.1.1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Authn/Authz</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>U.C.3.1.2</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>U.C.10.3.2, U.C.10.3.1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Authn/Authz</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>U.C.3.2.1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>U.C.7.5.1, U.C.8.*, U.C.10.3.1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Authn/Authz</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>U.C.3.3.1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Authn/Authz</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>U.C.3.4.1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Authn/Authz</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>U.C.3.5.1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Authn/Authz</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>U.C.3.6.1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Authn/Authz</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>U.C.4.1.1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>U.C.8.*, U.C.10.*</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Secure development</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>U.C.4.2.1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>U.C.8.*, U.C.9.3.1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Secure development</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>U.C.4.3.1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Secure development</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>U.C.4.4.1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>U.C.8.3.1, U.C.9.4.1, U.C.10.1.1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Secure development</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>U.C.4.5.1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>U.C.10.2.1, U.C.10.3.2, U.C.11.x</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Secure development</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>U.C.5.1.1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Governance / DPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>U.C.5.1.2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Governance / DPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>U.C.5.2.1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>U.C.10.2.1, U.C.10.3.2, U.C.11.x</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Governance / DPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>U.C.5.3.1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>All U.C.7-11</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Governance / DPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>U.C.5.4.1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>U.C.10.2.1, U.C.7.1.2</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Governance / DPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>U.C.5.5.1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>U.C.10.2.1, U.C.7.1.2</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Governance / DPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>U.C.5.6.1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>U.C.8.*, U.C.10.*</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Governance / DPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>U.C.6.1.1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>All U.C.7-11 (human-driven)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>U.C.6.2.1</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>U.C.7.5.1, U.C.10.3.1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>U.C.6.3.1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>U.C.7.1.1, U.C.7.1.2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Awareness</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>MUC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Misactor</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Threatens Functional UC(s)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Mitigated by Security UC(s)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MUC-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A-MIS-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>U.C.7.1.2, U.C.7.1.3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>U.C.3.1.1, U.C.3.1.2, U.C.2.4.1, U.C.3.5.1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Credential Stuffing Against Login</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MUC-02</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A-MIS-03</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>U.C.7.5.1, U.C.10.3.1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>U.C.3.2.1, U.C.3.5.1, U.C.5.1.2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Privilege Escalation via Invite/Roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MUC-03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A-MIS-01/A-MIS-03</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>U.C.8.1.2, U.C.8.2.1, U.C.8.3.1, U.C.8.1.1, U.C.10.1.1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>U.C.3.3.1, U.C.3.2.1, U.C.2.1.1, U.C.4.2.1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cross-Tenant Data Injection/Read</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MUC-04</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A-MIS-03</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>U.C.11.2.1, U.C.9.4.1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>U.C.1.3.1, U.C.1.5.1, U.C.2.4.2, U.C.3.5.1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Bulk Data Extraction via Export Endpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MUC-05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A-MIS-04</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>U.C.10.2.1, U.C.7.1.2</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>U.C.5.4.1, U.C.5.5.1, U.C.3.1.1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Compromised Third-Party Integration</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MUC-06</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A-MIS-02</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>All U.C.7-11 (data plane)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>U.C.3.1.2, U.C.3.2.1, U.C.3.5.1, U.C.2.4.1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Malicious Insider Exfiltration</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MUC-07</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A-MIS-01</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>U.C.8.3.1, All U.C.7-11 (availability)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>U.C.2.4.2, U.C.4.4.1, U.C.2.6.1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Board / Service DoS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MUC-08</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>A-MIS-01</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>U.C.9.3.1</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>U.C.2.4.1, U.C.3.5.1, U.C.4.2.1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Malicious Attachment Upload</t>
         </is>
       </c>
     </row>
@@ -9751,7 +10873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9860,7 +10982,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>UC L1 cards</t>
+          <t>UC L1 cards (security)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -9883,14 +11005,14 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>FR cards</t>
+          <t>Functional U.C.s (new)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C6" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -9899,21 +11021,21 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FROZEN per RULE_FREEZE.md §6</t>
+          <t>Sprint 6 product baseline</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NFR cards</t>
+          <t>Misuse cases (new)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C7" t="n">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -9922,21 +11044,21 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>FROZEN per RULE_FREEZE.md §7</t>
+          <t>Sprint 6 Sindre &amp; Opdahl</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>DN rows</t>
+          <t>Constrains edges</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C8" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -9945,21 +11067,21 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Doc 15 §4, 1:1 with CR</t>
+          <t>Sprint 6 security→functional bridge</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Gates</t>
+          <t>MUC→mitigation edges</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -9968,21 +11090,21 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Doc 16 §5, 1:1 with CR</t>
+          <t>Sprint 6 threat model</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PO/SO Goals</t>
+          <t>FR cards</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -9991,21 +11113,21 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>11 PO + 20 SO per RULE_FREEZE.md §2</t>
+          <t>FROZEN per RULE_FREEZE.md §6</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Nodes (Doc 14)</t>
+          <t>NFR cards</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C11" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -10014,21 +11136,21 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>17 TECH + 20 PROC + 12 ROLE</t>
+          <t>FROZEN per RULE_FREEZE.md §7</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Risks</t>
+          <t>DN rows</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C12" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -10037,21 +11159,21 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>FROZEN per RULE_FREEZE.md §7.1</t>
+          <t>Doc 15 §4, 1:1 with CR</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Threats</t>
+          <t>Gates</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C13" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -10060,21 +11182,21 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FROZEN per RULE_FREEZE.md §7.1</t>
+          <t>Doc 16 §5, 1:1 with CR</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Total Artefacts</t>
+          <t>PO/SO Goals</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>345</v>
+        <v>31</v>
       </c>
       <c r="C14" t="n">
-        <v>345</v>
+        <v>31</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -10083,21 +11205,21 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sum (CORPUS_LINKAGE.md §10 = 345)</t>
+          <t>11 PO + 20 SO per RULE_FREEZE.md §2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>KG Chains</t>
+          <t>Nodes (Doc 14)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="C15" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -10106,80 +11228,172 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>12 chains per KG_CHAINS.md §1</t>
+          <t>17 TECH + 20 PROC + 12 ROLE</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>KG Contamination nodes (F-S1-09)</t>
+          <t>Risks</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>14</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>REPORT</t>
-        </is>
+        <v>10</v>
+      </c>
+      <c r="C16" t="n">
+        <v>10</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>All KG-extraction artefacts (RULE_FREEZE.md §4)</t>
+          <t>FROZEN per RULE_FREEZE.md §7.1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>F-register OPEN (Sprint 1)</t>
+          <t>Threats</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>F-S1-01..07</t>
-        </is>
+        <v>38</v>
+      </c>
+      <c r="C17" t="n">
+        <v>38</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Orphan CR-D refs in legacy Phase 3</t>
+          <t>FROZEN per RULE_FREEZE.md §7.1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Total Artefacts</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>345</v>
+      </c>
+      <c r="C18" t="n">
+        <v>345</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sum (CORPUS_LINKAGE.md §10 = 345)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>KG Chains</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C19" t="n">
+        <v>12</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>12 chains per KG_CHAINS.md §1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>KG Contamination nodes (F-S1-09)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>14</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>REPORT</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>All KG-extraction artefacts (RULE_FREEZE.md §4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>F-register OPEN (Sprint 1)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>7</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>F-S1-01..07</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Orphan CR-D refs in legacy Phase 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>F-register CARRIED</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B22" t="n">
         <v>1</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>F-S1-08</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Doc 08 ↔ Doc 11 OBL drift</t>
         </is>

</xml_diff>

<commit_message>
[EXECUTOR] LANE NAMING Case_01: 18 UCs re-laned (17 PROC + 1 CAP), 509 refs single-pass; Doc20 v3.1 §6.1 freeze superseded (P7); xlsx regenerated; gate PASS
</commit_message>
<xml_diff>
--- a/02_CASES/Case_01_TinyTask_SaaS/03_PHASE3_DECOMPOSITION_RICH/22_Traceability_Matrix.xlsx
+++ b/02_CASES/Case_01_TinyTask_SaaS/03_PHASE3_DECOMPOSITION_RICH/22_Traceability_Matrix.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-26 15:30 UTC</t>
+          <t>2026-09-05 13:28 UTC</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U.C.1.1.1</t>
+          <t>PROC-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rights enforcement</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>U.C.1.1.2</t>
+          <t>PROC-02</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Rights enforcement</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>U.C.2.1.1</t>
+          <t>PROC-03</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Availability / release gating</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>U.C.2.3.1</t>
+          <t>PROC-04</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Availability / release gating</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>U.C.2.5.1</t>
+          <t>PROC-05</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Availability / release gating</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>U.C.3.4.1</t>
+          <t>PROC-06</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Authn/Authz</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>U.C.3.6.1</t>
+          <t>PROC-07</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Authn/Authz</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>U.C.4.1.1</t>
+          <t>PROC-08</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Secure development</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>U.C.4.5.1</t>
+          <t>PROC-09</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Secure development</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>U.C.5.1.1</t>
+          <t>PROC-10</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Governance / DPA</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>U.C.5.1.2</t>
+          <t>PROC-11</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Governance / DPA</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>U.C.5.2.1</t>
+          <t>PROC-12</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Governance / DPA</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>U.C.5.3.1</t>
+          <t>PROC-13</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Governance / DPA</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>U.C.5.4.1</t>
+          <t>PROC-14</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Governance / DPA</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>U.C.5.5.1</t>
+          <t>CAP-01</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Governance / DPA</t>
+          <t>Awareness</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>U.C.6.1.1</t>
+          <t>PROC-15</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>U.C.6.2.1</t>
+          <t>PROC-16</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>U.C.6.3.1</t>
+          <t>PROC-17</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>U.C.3.2.1, U.C.3.5.1, U.C.5.1.2</t>
+          <t>U.C.3.2.1, U.C.3.5.1, PROC-11</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>U.C.3.3.1, U.C.3.2.1, U.C.2.1.1, U.C.4.2.1</t>
+          <t>U.C.3.3.1, U.C.3.2.1, PROC-03, U.C.4.2.1</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>U.C.5.4.1, U.C.5.5.1, U.C.3.1.1</t>
+          <t>PROC-14, CAP-01, U.C.3.1.1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>U.C.1.1.1, U.C.1.2.1, U.C.1.3.1, U.C.1.4.1, U.C.1.5.1</t>
+          <t>PROC-01, U.C.1.2.1, U.C.1.3.1, U.C.1.4.1, U.C.1.5.1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>U.C.2.1.1, U.C.2.3.1, U.C.2.4.1, U.C.2.6.1, U.C.4.3.1, U.C.5.5.1</t>
+          <t>CAP-01, PROC-03, PROC-04, U.C.2.4.1, U.C.2.6.1, U.C.4.3.1</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>U.C.2.5.1, U.C.3.1.1, U.C.3.2.1, U.C.3.3.1, U.C.3.5.1, U.C.3.6.1</t>
+          <t>PROC-05, PROC-07, U.C.3.1.1, U.C.3.2.1, U.C.3.3.1, U.C.3.5.1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>U.C.2.1.1, U.C.2.2.1</t>
+          <t>PROC-03, U.C.2.2.1</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -3915,7 +3915,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>U.C.5.1.1, U.C.5.2.1, U.C.5.3.1, U.C.5.4.1</t>
+          <t>PROC-10, PROC-12, PROC-13, PROC-14</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -3985,7 +3985,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>U.C.4.5.1</t>
+          <t>PROC-09</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>U.C.4.1.1, U.C.4.2.1, U.C.4.3.1</t>
+          <t>PROC-08, U.C.4.2.1, U.C.4.3.1</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>U.C.6.1.1, U.C.6.2.1</t>
+          <t>PROC-15, PROC-16</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -6370,7 +6370,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>U.C.3.6.1</t>
+          <t>PROC-07</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -6427,7 +6427,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>U.C.3.4.1</t>
+          <t>PROC-06</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -6452,7 +6452,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>U.C.1.1.1</t>
+          <t>PROC-01</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -6608,7 +6608,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>U.C.2.1.1</t>
+          <t>PROC-03</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6638,7 +6638,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>U.C.2.1.1</t>
+          <t>PROC-03</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -6720,7 +6720,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>U.C.2.3.1</t>
+          <t>PROC-04</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>U.C.2.5.1</t>
+          <t>PROC-05</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -6798,7 +6798,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>U.C.4.1.1</t>
+          <t>PROC-08</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -6884,7 +6884,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>U.C.4.5.1</t>
+          <t>PROC-09</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -6936,12 +6936,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>U.C.5.1.1</t>
+          <t>PROC-10</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>U.C.5.2.1</t>
+          <t>PROC-12</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -6966,7 +6966,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>U.C.5.3.1</t>
+          <t>PROC-13</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -6992,7 +6992,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>U.C.5.4.1</t>
+          <t>PROC-14</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -7018,7 +7018,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>U.C.5.5.1</t>
+          <t>CAP-01</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -7044,12 +7044,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>U.C.6.1.1</t>
+          <t>PROC-15</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>U.C.6.2.1</t>
+          <t>PROC-16</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -7074,7 +7074,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>U.C.6.3.1</t>
+          <t>PROC-17</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U.C.1.1.1</t>
+          <t>PROC-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>U.C.1.1.2</t>
+          <t>PROC-02</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7386,7 +7386,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>U.C.2.1.1</t>
+          <t>PROC-03</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -7462,7 +7462,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>U.C.2.3.1</t>
+          <t>PROC-04</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>U.C.2.5.1</t>
+          <t>PROC-05</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -7804,7 +7804,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>U.C.3.4.1</t>
+          <t>PROC-06</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>U.C.3.6.1</t>
+          <t>PROC-07</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>U.C.4.1.1</t>
+          <t>PROC-08</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>U.C.4.5.1</t>
+          <t>PROC-09</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>U.C.5.1.1</t>
+          <t>PROC-10</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -8146,7 +8146,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>U.C.5.1.2</t>
+          <t>PROC-11</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -8184,7 +8184,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>U.C.5.2.1</t>
+          <t>PROC-12</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -8222,7 +8222,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>U.C.5.3.1</t>
+          <t>PROC-13</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>U.C.5.4.1</t>
+          <t>PROC-14</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -8298,7 +8298,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>U.C.5.5.1</t>
+          <t>CAP-01</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -8374,7 +8374,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>U.C.6.1.1</t>
+          <t>PROC-15</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -8412,7 +8412,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>U.C.6.2.1</t>
+          <t>PROC-16</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -8450,7 +8450,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>U.C.6.3.1</t>
+          <t>PROC-17</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">

</xml_diff>

<commit_message>
[EXECUTOR] F2 RENUMBER Case_01: U.C.x.y.z flattened → UC-01..40 (compliance 01..17 + product 18..40), two-phase, 20 files, xlsx+builder regenerated, 11 SVGs re-rendered; gates PASS (verify_rich 0, audit 100%, mermaid 192/192, smoke 16/16)
</commit_message>
<xml_diff>
--- a/02_CASES/Case_01_TinyTask_SaaS/03_PHASE3_DECOMPOSITION_RICH/22_Traceability_Matrix.xlsx
+++ b/02_CASES/Case_01_TinyTask_SaaS/03_PHASE3_DECOMPOSITION_RICH/22_Traceability_Matrix.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-05 13:28 UTC</t>
+          <t>2026-09-05 23:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>U.C.11.1.1, U.C.11.2.1, U.C.11.3.1</t>
+          <t>UC-38, UC-39, UC-40</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>U.C.11.1.1</t>
+          <t>UC-38</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1532,12 +1532,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>U.C.1.2.1</t>
+          <t>UC-01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>U.C.11.3.1</t>
+          <t>UC-40</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1552,12 +1552,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>U.C.1.3.1</t>
+          <t>UC-02</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>U.C.11.2.1</t>
+          <t>UC-39</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1572,12 +1572,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>U.C.1.4.1</t>
+          <t>UC-03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>U.C.7.1.1, U.C.11.1.1</t>
+          <t>UC-18, UC-38</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1592,12 +1592,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>U.C.1.5.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>U.C.11.2.1</t>
+          <t>UC-39</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>U.C.8.2.1, U.C.9.3.1</t>
+          <t>UC-25, UC-31</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1632,12 +1632,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>U.C.2.2.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1672,12 +1672,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>U.C.2.4.1</t>
+          <t>UC-06</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>U.C.8.2.1, U.C.9.3.1</t>
+          <t>UC-25, UC-31</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1692,12 +1692,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>U.C.2.4.2</t>
+          <t>UC-07</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1732,12 +1732,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>U.C.2.6.1</t>
+          <t>UC-08</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1752,12 +1752,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>U.C.3.1.1</t>
+          <t>UC-09</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>U.C.7.1.1, U.C.7.1.2, U.C.7.1.3, U.C.7.2.1, U.C.10.1.1</t>
+          <t>UC-18, UC-19, UC-20, UC-21, UC-34</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1772,12 +1772,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>U.C.3.1.2</t>
+          <t>UC-10</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>U.C.10.3.2, U.C.10.3.1</t>
+          <t>UC-37, UC-36</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1792,12 +1792,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>U.C.3.2.1</t>
+          <t>UC-11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>U.C.7.5.1, U.C.8.*, U.C.10.3.1</t>
+          <t>UC-22, UC-23, UC-24, UC-25, UC-26, UC-27, UC-28, UC-36</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1812,12 +1812,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>U.C.3.3.1</t>
+          <t>UC-12</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1852,12 +1852,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>U.C.3.5.1</t>
+          <t>UC-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>U.C.8.*, U.C.10.*</t>
+          <t>UC-23, UC-24, UC-25, UC-26, UC-27, UC-28, UC-34, UC-35, UC-36, UC-37</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1912,12 +1912,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>U.C.4.2.1</t>
+          <t>UC-14</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>U.C.8.*, U.C.9.3.1</t>
+          <t>UC-23, UC-24, UC-25, UC-26, UC-27, UC-28, UC-31</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1932,12 +1932,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>U.C.4.3.1</t>
+          <t>UC-15</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1952,12 +1952,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>U.C.4.4.1</t>
+          <t>UC-16</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>U.C.8.3.1, U.C.9.4.1, U.C.10.1.1</t>
+          <t>UC-28, UC-32, UC-34</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>U.C.10.2.1, U.C.10.3.2, U.C.11.x</t>
+          <t>UC-35, UC-37, UC-38, UC-39, UC-40</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>U.C.10.2.1, U.C.10.3.2, U.C.11.x</t>
+          <t>UC-35, UC-37, UC-38, UC-39, UC-40</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>All U.C.7-11</t>
+          <t>All UC-18..UC-40</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>U.C.10.2.1, U.C.7.1.2</t>
+          <t>UC-35, UC-19</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>U.C.10.2.1, U.C.7.1.2</t>
+          <t>UC-35, UC-19</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2112,12 +2112,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>U.C.5.6.1</t>
+          <t>UC-17</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>U.C.8.*, U.C.10.*</t>
+          <t>UC-23, UC-24, UC-25, UC-26, UC-27, UC-28, UC-34, UC-35, UC-36, UC-37</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>All U.C.7-11 (human-driven)</t>
+          <t>All UC-18..UC-40 (human-driven)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>U.C.7.5.1, U.C.10.3.1</t>
+          <t>UC-22, UC-36</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>U.C.7.1.1, U.C.7.1.2</t>
+          <t>UC-18, UC-19</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2203,8 +2203,8 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -2256,12 +2256,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>U.C.7.1.2, U.C.7.1.3</t>
+          <t>UC-19, UC-20</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>U.C.3.1.1, U.C.3.1.2, U.C.2.4.1, U.C.3.5.1</t>
+          <t>UC-09, UC-10, UC-06, UC-13</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2286,12 +2286,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>U.C.7.5.1, U.C.10.3.1</t>
+          <t>UC-22, UC-36</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>U.C.3.2.1, U.C.3.5.1, PROC-11</t>
+          <t>UC-11, UC-13, PROC-11</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2316,12 +2316,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>U.C.8.1.2, U.C.8.2.1, U.C.8.3.1, U.C.8.1.1, U.C.10.1.1</t>
+          <t>UC-24, UC-25, UC-28, UC-23, UC-34</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>U.C.3.3.1, U.C.3.2.1, PROC-03, U.C.4.2.1</t>
+          <t>UC-12, UC-11, PROC-03, UC-14</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2346,12 +2346,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>U.C.11.2.1, U.C.9.4.1</t>
+          <t>UC-39, UC-32</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>U.C.1.3.1, U.C.1.5.1, U.C.2.4.2, U.C.3.5.1</t>
+          <t>UC-02, UC-04, UC-07, UC-13</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2376,12 +2376,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>U.C.10.2.1, U.C.7.1.2</t>
+          <t>UC-35, UC-19</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>PROC-14, CAP-01, U.C.3.1.1</t>
+          <t>PROC-14, CAP-01, UC-09</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2406,12 +2406,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>All U.C.7-11 (data plane)</t>
+          <t>All UC-18..UC-40 (data plane)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>U.C.3.1.2, U.C.3.2.1, U.C.3.5.1, U.C.2.4.1</t>
+          <t>UC-10, UC-11, UC-13, UC-06</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2436,12 +2436,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>U.C.8.3.1, All U.C.7-11 (availability)</t>
+          <t>UC-28, All UC-18..UC-40 (availability)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>U.C.2.4.2, U.C.4.4.1, U.C.2.6.1</t>
+          <t>UC-07, UC-16, UC-08</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2466,12 +2466,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>U.C.9.3.1</t>
+          <t>UC-31</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>U.C.2.4.1, U.C.3.5.1, U.C.4.2.1</t>
+          <t>UC-06, UC-13, UC-14</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2500,7 +2500,7 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="51" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="47" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -2613,7 +2613,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>PROC-01, U.C.1.2.1, U.C.1.3.1, U.C.1.4.1, U.C.1.5.1</t>
+          <t>PROC-01, UC-01, UC-02, UC-03, UC-04</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CAP-01, PROC-03, PROC-04, U.C.2.4.1, U.C.2.6.1, U.C.4.3.1</t>
+          <t>CAP-01, PROC-03, PROC-04, UC-06, UC-08, UC-15</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>PROC-05, PROC-07, U.C.3.1.1, U.C.3.2.1, U.C.3.3.1, U.C.3.5.1</t>
+          <t>PROC-05, PROC-07, UC-09, UC-11, UC-12, UC-13</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>PROC-03, U.C.2.2.1</t>
+          <t>PROC-03, UC-05</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>U.C.1.6.1 (legacy), U.C.2.2.1</t>
+          <t>U.C.1.6.1 (legacy), UC-05</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>PROC-08, U.C.4.2.1, U.C.4.3.1</t>
+          <t>PROC-08, UC-14, UC-15</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -6226,8 +6226,8 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
@@ -6288,12 +6288,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>U.C.3.2.1</t>
+          <t>UC-11</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>U.C.3.5.1</t>
+          <t>UC-13</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -6318,7 +6318,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>U.C.3.1.1</t>
+          <t>UC-09</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -6344,7 +6344,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>U.C.3.3.1</t>
+          <t>UC-12</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -6396,7 +6396,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>U.C.3.5.1</t>
+          <t>UC-13</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -6422,7 +6422,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>U.C.3.1.1</t>
+          <t>UC-09</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6478,7 +6478,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>U.C.1.2.1</t>
+          <t>UC-01</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -6504,7 +6504,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>U.C.1.3.1</t>
+          <t>UC-02</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>U.C.1.4.1</t>
+          <t>UC-03</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>U.C.1.5.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>U.C.1.4.1</t>
+          <t>UC-03</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -6613,7 +6613,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>U.C.2.6.1</t>
+          <t>UC-08</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -6664,7 +6664,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>U.C.2.2.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -6695,7 +6695,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>U.C.2.2.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>U.C.2.4.1</t>
+          <t>UC-06</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -6803,12 +6803,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>U.C.4.2.1</t>
+          <t>UC-14</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>U.C.4.3.1</t>
+          <t>UC-15</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -6832,7 +6832,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>U.C.4.3.1</t>
+          <t>UC-15</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -6858,7 +6858,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>U.C.4.4.1</t>
+          <t>UC-16</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -7101,7 +7101,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -7234,7 +7234,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>U.C.1.2.1</t>
+          <t>UC-01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -7272,7 +7272,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>U.C.1.3.1</t>
+          <t>UC-02</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -7310,7 +7310,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>U.C.1.4.1</t>
+          <t>UC-03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>U.C.1.5.1</t>
+          <t>UC-04</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>U.C.2.2.1</t>
+          <t>UC-05</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -7500,7 +7500,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>U.C.2.4.1</t>
+          <t>UC-06</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -7538,7 +7538,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>U.C.2.4.2</t>
+          <t>UC-07</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -7614,7 +7614,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>U.C.2.6.1</t>
+          <t>UC-08</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>U.C.3.1.1</t>
+          <t>UC-09</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -7690,7 +7690,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>U.C.3.1.2</t>
+          <t>UC-10</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>U.C.3.2.1</t>
+          <t>UC-11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -7766,7 +7766,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>U.C.3.3.1</t>
+          <t>UC-12</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -7842,7 +7842,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>U.C.3.5.1</t>
+          <t>UC-13</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -7956,7 +7956,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>U.C.4.2.1</t>
+          <t>UC-14</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>U.C.4.3.1</t>
+          <t>UC-15</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -8032,7 +8032,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>U.C.4.4.1</t>
+          <t>UC-16</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>U.C.5.6.1</t>
+          <t>UC-17</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">

</xml_diff>